<commit_message>
Update Supplementary Table 1
</commit_message>
<xml_diff>
--- a/Supplementary Table 1 - Tools Used by Phase.xlsx
+++ b/Supplementary Table 1 - Tools Used by Phase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdagcc-my.sharepoint.com/personal/david_bradshaw_usda_gov/Documents/Documents/Manuscripts/UK1_Reverse_Vaccinology/GitHub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{575186B5-6A00-4A68-AF0E-B0240DBFC1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{575186B5-6A00-4A68-AF0E-B0240DBFC1FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF6D4383-C544-420C-AC44-950061CC8A75}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5976EEAC-27D5-4F09-91B6-0764888DA880}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5976EEAC-27D5-4F09-91B6-0764888DA880}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,18 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="123">
-  <si>
-    <t>Supplementary Table 1: Tools used by Phase</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="131">
   <si>
     <t>Phase</t>
   </si>
   <si>
     <t>Tool</t>
-  </si>
-  <si>
-    <t>Purpose</t>
   </si>
   <si>
     <t>Website</t>
@@ -76,9 +70,6 @@
     <t>Vaxign-ML</t>
   </si>
   <si>
-    <t>Antigencity Prediction</t>
-  </si>
-  <si>
     <t>Ong et al. (2020)</t>
   </si>
   <si>
@@ -98,9 +89,6 @@
     <t>SPAAN</t>
   </si>
   <si>
-    <t>Adhesion Propability</t>
-  </si>
-  <si>
     <t>Sachdeva et al. (2005)</t>
   </si>
   <si>
@@ -119,11 +107,6 @@
   <si>
     <t>BLAST+ (v.2.14.1)
 BLASTP</t>
-  </si>
-  <si>
-    <t>Similar Proteins
-Negative Homology with Hosts
-Positive Homology with Serovars</t>
   </si>
   <si>
     <t>https://blast.ncbi.nlm.nih.gov/Blast.cgi?PAGE=Proteins</t>
@@ -186,9 +169,6 @@
     <t>IEDB Immunogenicty</t>
   </si>
   <si>
-    <t>CTL Immunogencity Prediction</t>
-  </si>
-  <si>
     <t>http://tools.iedb.org/immunogenicity/</t>
   </si>
   <si>
@@ -213,18 +193,9 @@
 Evaluation</t>
   </si>
   <si>
-    <t>ANTIGENpro</t>
-  </si>
-  <si>
-    <t>Antigenicity Prediction</t>
-  </si>
-  <si>
     <t>http://scratch.proteomics.ics.uci.edu/</t>
   </si>
   <si>
-    <t>Cheng et al. (2005)</t>
-  </si>
-  <si>
     <t>ToxinPred2</t>
   </si>
   <si>
@@ -243,15 +214,9 @@
     <t>Solubility Prediction</t>
   </si>
   <si>
-    <t>Magnan et al. (2009)</t>
-  </si>
-  <si>
     <t>AllergenFP</t>
   </si>
   <si>
-    <t>Allergenicty Prediction</t>
-  </si>
-  <si>
     <t>https://ddg-pharmfac.net/AllergenFP/</t>
   </si>
   <si>
@@ -351,18 +316,6 @@
     <t>Laskowski et al. (1993)</t>
   </si>
   <si>
-    <t>ElliPro</t>
-  </si>
-  <si>
-    <t>Confirmational B-Cell Epitope Prediction</t>
-  </si>
-  <si>
-    <t>http://tools.iedb.org/ellipro/</t>
-  </si>
-  <si>
-    <t>Ponomarenko et al. (2008)</t>
-  </si>
-  <si>
     <t>ClusPro</t>
   </si>
   <si>
@@ -387,9 +340,6 @@
     <t>Abraham et al. (2015)</t>
   </si>
   <si>
-    <t>Jcat</t>
-  </si>
-  <si>
     <t>Codon Optimization</t>
   </si>
   <si>
@@ -418,6 +368,83 @@
   </si>
   <si>
     <t>Rapin et al. (2010)</t>
+  </si>
+  <si>
+    <t>Supplementary Table 1: Reverse vaccinology tools used by Phase</t>
+  </si>
+  <si>
+    <t>Purpose(s)</t>
+  </si>
+  <si>
+    <t>Protein Antigenicity Prediction</t>
+  </si>
+  <si>
+    <t>Adhesion Probability</t>
+  </si>
+  <si>
+    <t>Similar Proteins
+Negative Homology with Hosts
+Protein Positive Homology with Serovars</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Protein Antigenicity Prediction</t>
+  </si>
+  <si>
+    <t>CTL Immunogenicity Prediction</t>
+  </si>
+  <si>
+    <t>Epitope Antigenicity Prediction
+Overlapping Epitope Selection</t>
+  </si>
+  <si>
+    <t>Epitope Positive Homology with Serovars</t>
+  </si>
+  <si>
+    <t>MEVC Antigenicity Prediction</t>
+  </si>
+  <si>
+    <t>Allergenicity Prediction</t>
+  </si>
+  <si>
+    <t>SOLpro - Magnan et al. (2009)
+SCRATCH - Cheng et al. (2005)</t>
+  </si>
+  <si>
+    <t>PDBsum</t>
+  </si>
+  <si>
+    <t>Receptor-Ligand Interactions</t>
+  </si>
+  <si>
+    <t>https://www.ebi.ac.uk/thornton-srv/databases/pdbsum/</t>
+  </si>
+  <si>
+    <t>Laskowski et al. (2018)</t>
+  </si>
+  <si>
+    <t>JCat</t>
+  </si>
+  <si>
+    <t>gBlocks™ Gene Fragments Entry Tool</t>
+  </si>
+  <si>
+    <t>Nucleotide Sequence Complexity</t>
+  </si>
+  <si>
+    <t>https://www.idtdna.com/SciTools</t>
+  </si>
+  <si>
+    <t>Owczarzy et al. (2008)</t>
+  </si>
+  <si>
+    <t>Codon Optimization Tool</t>
+  </si>
+  <si>
+    <t>Codon Optimization
+Nucleotide Sequence Complexity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEVC is multiepitope vaccine construct. </t>
   </si>
 </sst>
 </file>
@@ -433,13 +460,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -714,111 +743,109 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1151,535 +1178,584 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD86AC9-9B8F-4C0B-AB92-15DC77886D7C}">
-  <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.85546875" style="34" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.7109375" style="33" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" style="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="16" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="49.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.28515625" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="6" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="C3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="10" t="s">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="12"/>
+      <c r="B4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="C4" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14" t="s">
+    <row r="5" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A5" s="12"/>
+      <c r="B5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="16" t="s">
+      <c r="D5" s="14" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14" t="s">
+      <c r="E5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="15" t="s">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="12"/>
+      <c r="B6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="C6" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="16" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="12"/>
+      <c r="B7" s="13" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="D7" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="16" t="s">
+      <c r="E7" s="15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14" t="s">
+    <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="12"/>
+      <c r="B8" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C8" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="E8" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="16" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="17"/>
+      <c r="B9" s="18" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="15" t="s">
+      <c r="C9" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="E9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="14" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="B10" s="22" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18"/>
-      <c r="B9" s="19" t="s">
+      <c r="C10" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="19" t="s">
+      <c r="D10" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E10" s="24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="25"/>
+      <c r="B11" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="C11" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="D11" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="E11" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="25" t="s">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="25"/>
+      <c r="B12" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A13" s="29"/>
+      <c r="B13" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="29"/>
+      <c r="B14" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="29"/>
+      <c r="B15" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="29"/>
+      <c r="B16" s="13" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="26"/>
-      <c r="B11" s="14" t="s">
+      <c r="C16" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="D16" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="E16" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="16" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="26"/>
-      <c r="B12" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="14" t="s">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="B17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="25"/>
+      <c r="B18" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A19" s="25"/>
+      <c r="B19" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="13" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="23.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="27"/>
-      <c r="B14" s="28" t="s">
+      <c r="E19" s="16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="25"/>
+      <c r="B20" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C20" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D20" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="30" t="s">
+      <c r="E20" s="15" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="26"/>
-      <c r="B16" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="26"/>
-      <c r="B17" s="14" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="25"/>
+      <c r="B21" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C21" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D21" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E21" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="26"/>
-      <c r="B18" s="14" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="25"/>
+      <c r="B22" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C22" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E18" s="16" t="s">
+      <c r="D22" s="13" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="26"/>
-      <c r="B19" s="14" t="s">
+      <c r="E22" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="15" t="s">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="25"/>
+      <c r="B23" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="C23" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="D23" s="13" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="26"/>
-      <c r="B20" s="14" t="s">
+      <c r="E23" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C20" s="15" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="25"/>
+      <c r="B24" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="C24" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="E20" s="16" t="s">
+      <c r="D24" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="26"/>
-      <c r="B21" s="14" t="s">
+      <c r="E24" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="15" t="s">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="25"/>
+      <c r="B25" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="C25" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="16" t="s">
+      <c r="D25" s="13" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="26"/>
-      <c r="B22" s="14" t="s">
+      <c r="E25" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="15" t="s">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="25"/>
+      <c r="B26" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="25"/>
+      <c r="B27" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="25"/>
+      <c r="B28" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="25"/>
+      <c r="B29" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="C29" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="D29" s="13" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="26"/>
-      <c r="B23" s="14" t="s">
+      <c r="E29" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D23" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="26"/>
-      <c r="B24" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="26"/>
-      <c r="B25" s="14" t="s">
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="25"/>
+      <c r="B30" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C30" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D30" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="E25" s="16" t="s">
+      <c r="E30" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="26"/>
-      <c r="B26" s="14" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="25"/>
+      <c r="B31" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="25"/>
+      <c r="B32" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="D26" s="14" t="s">
+      <c r="C32" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="E26" s="16" t="s">
+      <c r="D32" s="13" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="26"/>
-      <c r="B27" s="14" t="s">
+      <c r="E32" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="C27" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="E27" s="16" t="s">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="25"/>
+      <c r="B33" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="26"/>
-      <c r="B28" s="14" t="s">
+      <c r="D33" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="E28" s="16" t="s">
+      <c r="E33" s="15" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="26"/>
-      <c r="B29" s="14" t="s">
+    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A34" s="25"/>
+      <c r="B34" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D34" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A35" s="25"/>
+      <c r="B35" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="25"/>
+      <c r="B36" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C36" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D36" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="E29" s="16" t="s">
+      <c r="E36" s="15" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="26"/>
-      <c r="B30" s="14" t="s">
+    <row r="37" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="32"/>
+      <c r="B37" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C37" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D37" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="E37" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="E30" s="16" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="26"/>
-      <c r="B31" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="E31" s="16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="26"/>
-      <c r="B32" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="E32" s="16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="26"/>
-      <c r="B33" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="E33" s="16" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="32"/>
-      <c r="B34" s="19" t="s">
-        <v>120</v>
-      </c>
-      <c r="C34" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="D34" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>122</v>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:A9"/>
-    <mergeCell ref="A10:A14"/>
-    <mergeCell ref="A15:A34"/>
+    <mergeCell ref="A10:A16"/>
+    <mergeCell ref="A17:A37"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="D34" r:id="rId1" xr:uid="{276FE397-1F82-4F65-AB81-9F3E2A0DC0CD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>